<commit_message>
Organized filters in categories
</commit_message>
<xml_diff>
--- a/RoleFinder/job profiles.xlsx
+++ b/RoleFinder/job profiles.xlsx
@@ -655,7 +655,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2708" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2708" uniqueCount="154">
   <si>
     <t xml:space="preserve">מחלקה</t>
   </si>
@@ -729,7 +729,7 @@
     <t xml:space="preserve">ניסיון באינטגרציה </t>
   </si>
   <si>
-    <t xml:space="preserve">גר/ה רחוק בכרמיאל או נהריה </t>
+    <t xml:space="preserve">גר/ה רחוק בכרמיאל/נהריה </t>
   </si>
   <si>
     <t xml:space="preserve">רגישות לחומרים </t>
@@ -849,7 +849,7 @@
     <t xml:space="preserve">25-50</t>
   </si>
   <si>
-    <t xml:space="preserve">בזריזה </t>
+    <t xml:space="preserve">בתנועה </t>
   </si>
   <si>
     <t xml:space="preserve">38-40</t>
@@ -1111,6 +1111,9 @@
   </si>
   <si>
     <t xml:space="preserve">עם מיכרוסקופ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בתנועה</t>
   </si>
   <si>
     <t xml:space="preserve">20-35 </t>
@@ -10698,7 +10701,7 @@
       </c>
       <c r="D6" s="102"/>
       <c r="E6" s="95" t="s">
-        <v>64</v>
+        <v>152</v>
       </c>
       <c r="F6" s="95" t="s">
         <v>95</v>
@@ -10786,7 +10789,7 @@
     </row>
     <row r="9" customFormat="false" ht="32" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="105" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C9" s="100" t="s">
         <v>94</v>

</xml_diff>